<commit_message>
Refactor converter function to include sheet_name parameter and update related calls; add timestamp handling in Person class; create new utility functions and files for better data management.
</commit_message>
<xml_diff>
--- a/svar_klubbklar_26_27.xlsx
+++ b/svar_klubbklar_26_27.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fa017e0d854f10e/Dokumenter/NTNUI Klubbklær/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fa017e0d854f10e/Dokumenter/NTNUI Klubbklær/NTNUI-klubbklar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_1BCAB5A55B506C0E8DD0F04648BD99EA98F779CE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8773FEB4-3F62-4A74-A115-F09E7A3B3D44}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="11_1BCAB5A55B506C0E8DD0F04648BD99EA98F779CE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FAEBD3D-E706-49BC-A2DE-0EEB9FB31C28}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1700" yWindow="1700" windowWidth="2370" windowHeight="560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="5780" yWindow="5780" windowWidth="2370" windowHeight="560" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Skjemasvar 1" sheetId="1" r:id="rId1"/>
@@ -1497,7 +1497,7 @@
     </row>
     <row r="2" spans="1:70" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>46255.518463553242</v>
+        <v>46255.518460648149</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>64</v>

</xml_diff>